<commit_message>
Links: state what the fixture can and cannot show, make the week-one link audit the gate for Q1 order
Adds partial correlations (age vs drop with links held constant 0.80;
links vs drop with age held constant -0.07) to the analysis, and
replaces 'links are not the problem' with the open link hypotheses,
the tests that settle them, and what changes in the plan if they hit.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015LEzkrfcXznaX9ERkNGL27
</commit_message>
<xml_diff>
--- a/SEO_003_audit_and_refresh_model.xlsx
+++ b/SEO_003_audit_and_refresh_model.xlsx
@@ -280,7 +280,7 @@
     <t xml:space="preserve">weak, could be chance</t>
   </si>
   <si>
-    <t xml:space="preserve">No. The four pages with 50+ referring domains (84, 74, 61, 52) all fell. The two gainers have 26 and 11. Links explain where pages sit, not why they moved. Without the dated URLs: -0.28, could be chance.</t>
+    <t xml:space="preserve">No. The four pages with 50+ referring domains (84, 74, 61, 52) all fell, and they fell the least (2 to 5 places). The two gainers have 26 and 11. Once page age is held constant, link counts add nothing (partial correlation -0.07; age with links held constant: 0.80). What this file cannot see: link quality, links lost during the year, or competitors out-building us. Quietly neutralized links would look like the same slow slide on the head terms. The week-one audit (new and lost by month, anchors, DR spread, manual actions report) settles it and decides the order of Q1.</t>
   </si>
   <si>
     <t xml:space="preserve">referring domains vs positions lost</t>
@@ -2284,7 +2284,7 @@
     <t xml:space="preserve">our domain (fill from Ahrefs in week one)</t>
   </si>
   <si>
-    <t xml:space="preserve">[Observed] Ramp nets about 340 new referring main domains a month and the pace roughly doubled from the first half to the second. Brex nets about 165. A $4,000 a month digital PR line will not match that on volume, so our links go to the handful of pages that convert or hold the head terms. The week-one link audit also looks for spikes in our own pace that line up with ranking drops (bought links, scraped links) before any disavow decision.</t>
+    <t xml:space="preserve">[Observed] Ramp nets about 340 new referring main domains a month and the pace roughly doubled from the first half to the second. Brex nets about 165. A $4,000 a month digital PR line will not match that on volume, so our links go to the handful of pages that convert or hold the head terms. The week-one link audit looks for spikes or drops in our own pace that line up with ranking changes, exact-match anchors, low-quality domains and any manual action. If it finds a problem, links move to the front of Q1 and the refresh program slows until it is dealt with.</t>
   </si>
   <si>
     <t xml:space="preserve">Click-through rate by Google position</t>

</xml_diff>

<commit_message>
Month-12 targets as low/base/stretch scenarios; scaled sample input labeled as a scenario assumption; tighter prose
- Targets_Month_12 now carries three scenarios (101K / 117K / 136K;
  1.5x / 2.2x / 3x conversions) with the head-term scaling called out
  as a scenario assumption that week-one Search Console data replaces.
- Removed the unsupported DR 62 line and the unevidenced past-work
  anecdote (and its Tier 0 evidence row).
- Copy-edit pass for concision; no numbers or claims removed.
- Deck slide 12 shows the three scenarios.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015LEzkrfcXznaX9ERkNGL27
</commit_message>
<xml_diff>
--- a/SEO_003_audit_and_refresh_model.xlsx
+++ b/SEO_003_audit_and_refresh_model.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1453" uniqueCount="758">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="762">
   <si>
     <t xml:space="preserve">SEO recovery plan: audit and refresh model</t>
   </si>
@@ -70,7 +70,7 @@
     <t xml:space="preserve">7. Budget: the $15,000 a month split, and how many posts that buys.</t>
   </si>
   <si>
-    <t xml:space="preserve">8. Targets_Month_12: the month-12 traffic and conversion targets with every assumption in an editable cell.</t>
+    <t xml:space="preserve">8. Targets_Month_12: low, base and stretch month-12 targets for traffic and conversions, every assumption in an editable cell.</t>
   </si>
   <si>
     <t xml:space="preserve">Evidence sheets, for when you want to check a number: Data_To_Request (what we ask for in week one), Live_SERPs (who ranks today), Competitors (Ramp and Brex footprint and link pace), Ref_CTR_Curve (the click-through curve used in Page_Triage).</t>
@@ -1294,7 +1294,7 @@
     <t xml:space="preserve">Sprint 4: reserve for whatever the data says (field vitals, schema, the next template).</t>
   </si>
   <si>
-    <t xml:space="preserve">Organic conversions about 2x baseline. Traffic 115K to 120K. 140K is not promised: the AI Overview on the head terms and the two expired URLs cap what the old pages can return; anything above comes from new clusters and templates.</t>
+    <t xml:space="preserve">Base case: organic conversions about 2x baseline, traffic about 117K (low about 101K, stretch about 136K). 140K sits above the stretch case: the AI Overview on the head terms and the two expired URLs cap what the old pages can return; anything above comes from new clusters and templates.</t>
   </si>
   <si>
     <t xml:space="preserve">The five 90-day indicators</t>
@@ -1474,15 +1474,27 @@
     <t xml:space="preserve">50 posts in 6 months in the brief. We cannot match it on new posts (48 a year). Refreshes and consolidations are where our effort goes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Month-12 targets: traffic and conversions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What this sheet tells you: a labeled projection, not a forecast. Every yellow cell is an assumption you can change and the targets update.</t>
+    <t xml:space="preserve">Month-12 targets: three scenarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What this sheet tells you: a labeled projection, not a forecast. Low, base and stretch cases side by side. Every yellow cell is an assumption you can change and the three results update.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caveat that applies to every row below: the head-term share of loss (46%) comes from an 18-page sample of the biggest pages, and the written answer says not to scale that sample to the site. This sheet does scale it, as a scenario input only, so the targets have a shape. Search Console data in week one replaces the scaled input with the real one.</t>
   </si>
   <si>
     <t xml:space="preserve">Assumption</t>
   </si>
   <si>
+    <t xml:space="preserve">Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stretch</t>
+  </si>
+  <si>
     <t xml:space="preserve">Where it comes from</t>
   </si>
   <si>
@@ -1501,13 +1513,13 @@
     <t xml:space="preserve">Traffic the head-term pages lost across the site in 12 months</t>
   </si>
   <si>
-    <t xml:space="preserve">Head terms (cause B) are 46% of the sample's loss. Site loss is 55,000 (140K to 85K). 46% of 55,000 is about 25,000.</t>
+    <t xml:space="preserve">Scenario input. Base takes the sample's 46% head-term share of a 55,000 site loss (140K to 85K). Low and stretch bracket it. Replace with Search Console page data.</t>
   </si>
   <si>
     <t xml:space="preserve">Share of that we can win back while an AI Overview sits above #1</t>
   </si>
   <si>
-    <t xml:space="preserve">Ahrefs, February 2026, 300,000 keywords: 58% lower click rate for the top result when an AI Overview appears. Winning back rank returns under half the old clicks.</t>
+    <t xml:space="preserve">Ahrefs, February 2026, 300,000 keywords: 58% lower click rate for the top result when an AI Overview appears. Winning back rank returns under half the old clicks in the base case.</t>
   </si>
   <si>
     <t xml:space="preserve">Traffic lift on a refreshed non-head page, 6 months after the refresh</t>
@@ -1531,19 +1543,19 @@
     <t xml:space="preserve">Traffic won back by making the dated URLs evergreen (monthly, by month 12)</t>
   </si>
   <si>
-    <t xml:space="preserve">Two URLs peaked at 12,900 combined. Government and IRS own both SERPs now, so assume a third comes back.</t>
+    <t xml:space="preserve">Two URLs peaked at 12,900 combined. Government and IRS own both SERPs now.</t>
   </si>
   <si>
     <t xml:space="preserve">Traffic from new content by month 12 (48 new posts plus the comparison hub)</t>
   </si>
   <si>
-    <t xml:space="preserve">About 190 visits a post at month 12, in line with the spend management page's 650 at under a year old.</t>
+    <t xml:space="preserve">Base is about 190 visits a post at month 12, in line with the spend management page's 650 at under a year old.</t>
   </si>
   <si>
     <t xml:space="preserve">Conversion lift from CTAs, the comparison hub and templates (multiplier on conversions per visit)</t>
   </si>
   <si>
-    <t xml:space="preserve">Comparison pages convert at 10 to 13 per 1,000 visits against a blended 1.85. Moving a tenth of visits to that path and fixing CTAs on the top 6 pages.</t>
+    <t xml:space="preserve">Comparison pages convert at 10 to 13 per 1,000 visits against a blended 1.85. Base moves a tenth of visits to that path and fixes CTAs on the top 6 pages.</t>
   </si>
   <si>
     <t xml:space="preserve">Month-12 projection</t>
@@ -1576,7 +1588,7 @@
     <t xml:space="preserve">Projected organic conversions, month 12 (index, start = 100)</t>
   </si>
   <si>
-    <t xml:space="preserve">Reading: with these assumptions the site lands near 115K to 120K rather than 140K, because the head-term pages sit under an AI Overview and the two expired URLs are government-owned queries now. Conversions can roughly double because the conversion path (comparison hub, templates, CTAs) is where the upside is. The Q1 holdout replaces the assumed refresh lift with a measured one.</t>
+    <t xml:space="preserve">Reading: low about 101K, base about 117K, stretch about 136K. The brief's 140K sits above the stretch case, because the head-term pages sit under an AI Overview and the two expired URLs are government-owned queries now. Conversions land between about 1.5x and 3x, base about 2.2x, because the conversion path (comparison hub, templates, CTAs) is where the upside is. The base case is a scenario, not a promise: the Q1 holdout replaces the refresh lift, and week-one Search Console data replaces the scaled head-term loss.</t>
   </si>
   <si>
     <t xml:space="preserve">What we ask for in week one</t>
@@ -3130,7 +3142,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3140,7 +3152,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3158,22 +3170,22 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>344</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3181,19 +3193,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3201,19 +3213,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3221,19 +3233,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3241,19 +3253,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3261,19 +3273,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3281,19 +3293,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3301,19 +3313,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3321,19 +3333,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3341,19 +3353,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
     </row>
   </sheetData>
@@ -3393,7 +3405,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3408,7 +3420,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3436,1533 +3448,1533 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>116</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H5" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H6" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="K6" s="19"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H7" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B8" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H8" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I8" s="19" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="I9" s="19" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="J9" s="19" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="I10" s="19" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="J10" s="19" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="K10" s="19"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H11" s="19" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="I11" s="19" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="I12" s="19" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="K12" s="19"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B13" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="I13" s="19" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="J13" s="19" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="K13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B14" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H14" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I14" s="19" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="J14" s="19" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="K14" s="19" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B15" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H15" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I15" s="19" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="J15" s="19" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="K15" s="19" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B16" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H16" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I16" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="K16" s="19" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H17" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I17" s="19" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="J17" s="19" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="K17" s="19" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B18" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H18" s="19" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="I18" s="19" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="J18" s="19" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="K18" s="19"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="I19" s="19" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="J19" s="19" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="K19" s="19"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B20" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H20" s="19" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="I20" s="19" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="J20" s="19" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="K20" s="19" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B21" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="I21" s="19" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="J21" s="19" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="K21" s="19"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B22" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H22" s="19" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="I22" s="19" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="J22" s="19" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="K22" s="19"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B23" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H23" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I23" s="19" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="J23" s="19" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="K23" s="19" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B24" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H24" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I24" s="19" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="J24" s="19" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="K24" s="19"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B25" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H25" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I25" s="19" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="J25" s="19" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="K25" s="19"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H26" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I26" s="19" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="J26" s="19" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="K26" s="19"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="I27" s="19" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="J27" s="19" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="K27" s="19"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="I28" s="19" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="J28" s="19" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="K28" s="19"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B29" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="I29" s="19" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="J29" s="19" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="K29" s="19" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E30" s="19" t="s">
+        <v>633</v>
+      </c>
+      <c r="F30" s="19" t="s">
+        <v>581</v>
+      </c>
+      <c r="G30" s="19" t="s">
+        <v>582</v>
+      </c>
+      <c r="H30" s="19" t="s">
+        <v>605</v>
+      </c>
+      <c r="I30" s="19" t="s">
         <v>629</v>
       </c>
-      <c r="F30" s="19" t="s">
-        <v>577</v>
-      </c>
-      <c r="G30" s="19" t="s">
-        <v>578</v>
-      </c>
-      <c r="H30" s="19" t="s">
-        <v>601</v>
-      </c>
-      <c r="I30" s="19" t="s">
-        <v>625</v>
-      </c>
       <c r="J30" s="19" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="K30" s="19" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="I31" s="19" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="J31" s="19" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="K31" s="19" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B32" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H32" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I32" s="19" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="J32" s="19" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="K32" s="19" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B33" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F33" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H33" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I33" s="19" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="J33" s="19" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="K33" s="19"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B34" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H34" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I34" s="19" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="J34" s="19" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="K34" s="19"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B35" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H35" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I35" s="19" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="J35" s="19" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="K35" s="19"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B36" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="I36" s="19" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="J36" s="19" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="K36" s="19" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B37" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="I37" s="19" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="J37" s="19" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="K37" s="19"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B38" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G38" s="19" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="I38" s="19" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="J38" s="19" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="K38" s="19"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B39" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E39" s="19" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="I39" s="19" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="J39" s="19" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="K39" s="19"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B40" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="I40" s="19" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="J40" s="19" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="K40" s="19"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B41" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H41" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I41" s="19" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="J41" s="19" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="K41" s="19"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B42" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H42" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I42" s="19" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="J42" s="19" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="K42" s="19" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B43" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D43" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E43" s="19" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H43" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I43" s="19" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="J43" s="19" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="K43" s="19"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B44" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D44" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E44" s="19" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H44" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I44" s="19" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="J44" s="19" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="K44" s="19" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B45" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E45" s="19" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="I45" s="19" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="J45" s="19" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="K45" s="19" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B46" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D46" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="I46" s="19" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="J46" s="19" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="K46" s="19" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B47" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E47" s="19" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G47" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="I47" s="19" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="J47" s="19" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="K47" s="19" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B48" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D48" s="19" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F48" s="19" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="G48" s="19" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="I48" s="19" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="J48" s="19" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="K48" s="19" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4980,7 +4992,7 @@
     </row>
     <row r="50" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="B50" s="14"/>
       <c r="C50" s="14"/>
@@ -5008,7 +5020,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -5023,7 +5035,7 @@
     </row>
     <row r="53" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -5038,7 +5050,7 @@
     </row>
     <row r="54" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="B54" s="14"/>
       <c r="C54" s="14"/>
@@ -5053,7 +5065,7 @@
     </row>
     <row r="55" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="B55" s="14"/>
       <c r="C55" s="14"/>
@@ -5068,7 +5080,7 @@
     </row>
     <row r="56" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
@@ -5083,7 +5095,7 @@
     </row>
     <row r="57" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
@@ -5098,7 +5110,7 @@
     </row>
     <row r="58" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="B58" s="14"/>
       <c r="C58" s="14"/>
@@ -5153,7 +5165,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5172,7 +5184,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -5191,7 +5203,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -5210,66 +5222,66 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="F5" s="20" t="n">
         <v>2026</v>
@@ -5304,19 +5316,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="F6" s="20" t="n">
         <v>2026</v>
@@ -5351,19 +5363,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="F7" s="20" t="n">
         <v>2026</v>
@@ -5398,19 +5410,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="F8" s="20" t="n">
         <v>2026</v>
@@ -5445,19 +5457,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="F9" s="20" t="n">
         <v>2026</v>
@@ -5492,19 +5504,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="F10" s="20" t="n">
         <v>2026</v>
@@ -5539,7 +5551,7 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
@@ -5575,7 +5587,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -5594,40 +5606,40 @@
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
@@ -5635,19 +5647,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="F15" s="20" t="n">
         <v>8563</v>
@@ -5677,19 +5689,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="F16" s="20" t="n">
         <v>5382</v>
@@ -5719,19 +5731,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="F17" s="20" t="n">
         <v>4433</v>
@@ -5761,19 +5773,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="F18" s="20" t="n">
         <v>15000</v>
@@ -5803,19 +5815,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="F19" s="20" t="n">
         <v>6760</v>
@@ -5845,19 +5857,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="F20" s="20" t="n">
         <v>13667</v>
@@ -5887,19 +5899,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="F21" s="20" t="n">
         <v>31476</v>
@@ -5929,19 +5941,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="F22" s="20" t="n">
         <v>14045</v>
@@ -5971,19 +5983,19 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="F23" s="20" t="n">
         <v>36536</v>
@@ -6013,16 +6025,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E24" s="19" t="s">
         <v>111</v>
@@ -6055,19 +6067,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="F25" s="20" t="n">
         <v>47344</v>
@@ -6097,19 +6109,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="F26" s="20" t="n">
         <v>26473</v>
@@ -6139,19 +6151,19 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="F27" s="20" t="n">
         <v>14994</v>
@@ -6181,19 +6193,19 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="F28" s="20" t="n">
         <v>3225</v>
@@ -6223,19 +6235,19 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="F29" s="20" t="n">
         <v>4345</v>
@@ -6265,19 +6277,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>4418</v>
@@ -6307,19 +6319,19 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>6808</v>
@@ -6349,19 +6361,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>10232</v>
@@ -6391,19 +6403,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>11650</v>
@@ -6433,19 +6445,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>11323</v>
@@ -6475,19 +6487,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>18043</v>
@@ -6517,19 +6529,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C36" s="19" t="s">
+        <v>744</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>745</v>
+      </c>
+      <c r="E36" s="19" t="s">
         <v>740</v>
-      </c>
-      <c r="D36" s="19" t="s">
-        <v>741</v>
-      </c>
-      <c r="E36" s="19" t="s">
-        <v>736</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>14414</v>
@@ -6559,16 +6571,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E37" s="19" t="s">
         <v>111</v>
@@ -6601,19 +6613,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D38" s="19" t="s">
+        <v>745</v>
+      </c>
+      <c r="E38" s="19" t="s">
         <v>741</v>
-      </c>
-      <c r="E38" s="19" t="s">
-        <v>737</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>22928</v>
@@ -6643,19 +6655,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E39" s="19" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>32985</v>
@@ -6685,19 +6697,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>17453</v>
@@ -6744,7 +6756,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -6763,25 +6775,25 @@
     </row>
     <row r="43" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
@@ -6794,7 +6806,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="B44" s="16" t="n">
         <f aca="false">SUM(J15:J26)</f>
@@ -6831,7 +6843,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="B45" s="16" t="n">
         <f aca="false">SUM(J28:J39)</f>
@@ -6868,7 +6880,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="17" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -6904,7 +6916,7 @@
     </row>
     <row r="48" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="B48" s="14"/>
       <c r="C48" s="14"/>
@@ -6953,7 +6965,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6961,7 +6973,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -6975,16 +6987,16 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>403</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6995,10 +7007,10 @@
         <v>0.398</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7009,7 +7021,7 @@
         <v>0.187</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D6" s="10"/>
     </row>
@@ -7021,7 +7033,7 @@
         <v>0.102</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D7" s="10"/>
     </row>
@@ -7033,7 +7045,7 @@
         <v>0.072</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D8" s="10"/>
     </row>
@@ -7045,7 +7057,7 @@
         <v>0.051</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D9" s="10"/>
     </row>
@@ -7057,7 +7069,7 @@
         <v>0.044</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D10" s="10"/>
     </row>
@@ -7069,7 +7081,7 @@
         <v>0.03</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D11" s="10"/>
     </row>
@@ -7081,7 +7093,7 @@
         <v>0.021</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D12" s="10"/>
     </row>
@@ -7093,7 +7105,7 @@
         <v>0.019</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D13" s="10"/>
     </row>
@@ -7105,7 +7117,7 @@
         <v>0.016</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="D14" s="10"/>
     </row>
@@ -7120,7 +7132,7 @@
         <v>454</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11957,12 +11969,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="80"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11972,6 +11985,8 @@
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -11980,165 +11995,237 @@
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
+        <v>482</v>
+      </c>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>296</v>
+        <v>484</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F4" s="6" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>85000</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="18" t="n">
+        <v>85000</v>
+      </c>
+      <c r="D5" s="18" t="n">
+        <v>85000</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>442</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F5" s="10" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>454</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F6" s="10" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="B7" s="18" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C7" s="18" t="n">
         <v>25000</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="18" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>494</v>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>490</v>
-      </c>
-      <c r="B8" s="36" t="n">
+      <c r="F8" s="10" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>496</v>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>498</v>
+      </c>
+      <c r="B10" s="36" t="n">
         <v>0.4</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C10" s="36" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>492</v>
-      </c>
-      <c r="B9" s="36" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>454</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>494</v>
-      </c>
-      <c r="B10" s="36" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F10" s="10" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="B11" s="36" t="n">
         <v>0.25</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="36" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D11" s="10" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F11" s="10" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="B12" s="18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C12" s="18" t="n">
         <v>4000</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="18" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D12" s="10" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F12" s="10" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B13" s="18" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>9000</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="18" t="n">
+        <v>14000</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D13" s="10" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F13" s="10" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="B14" s="36" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C14" s="36" t="n">
         <v>1.6</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="36" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D14" s="10" t="s">
-        <v>503</v>
+      <c r="F14" s="10" t="s">
+        <v>507</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12146,147 +12233,238 @@
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>505</v>
-      </c>
-      <c r="B17" s="16" t="n">
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>509</v>
+      </c>
+      <c r="B18" s="16" t="n">
         <f aca="false">B5</f>
         <v>85000</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C18" s="16" t="n">
+        <f aca="false">C5</f>
+        <v>85000</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <f aca="false">D5</f>
+        <v>85000</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>442</v>
       </c>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>506</v>
-      </c>
-      <c r="B18" s="16" t="n">
-        <f aca="false">B7*B8</f>
-        <v>10000</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="D18" s="2"/>
+      <c r="F18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="B19" s="16" t="n">
-        <f aca="false">B5*(1-B11)*B10*B9</f>
-        <v>8606.25</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="D19" s="2"/>
+        <f aca="false">B7*B8</f>
+        <v>5000</v>
+      </c>
+      <c r="C19" s="16" t="n">
+        <f aca="false">C7*C8</f>
+        <v>10000</v>
+      </c>
+      <c r="D19" s="16" t="n">
+        <f aca="false">D7*D8</f>
+        <v>16500</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="F19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B20" s="16" t="n">
-        <f aca="false">B12</f>
-        <v>4000</v>
-      </c>
-      <c r="C20" s="7" t="s">
+        <f aca="false">B5*(1-B11)*B10*B9</f>
+        <v>3825</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <f aca="false">C5*(1-C11)*C10*C9</f>
+        <v>8606.25</v>
+      </c>
+      <c r="D20" s="16" t="n">
+        <f aca="false">D5*(1-D11)*D10*D9</f>
+        <v>14343.75</v>
+      </c>
+      <c r="E20" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D20" s="2"/>
+      <c r="F20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B21" s="16" t="n">
+        <f aca="false">B12</f>
+        <v>2000</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <f aca="false">C12</f>
+        <v>4000</v>
+      </c>
+      <c r="D21" s="16" t="n">
+        <f aca="false">D12</f>
+        <v>6000</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="F21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>513</v>
+      </c>
+      <c r="B22" s="16" t="n">
         <f aca="false">B13</f>
+        <v>5000</v>
+      </c>
+      <c r="C22" s="16" t="n">
+        <f aca="false">C13</f>
         <v>9000</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="D22" s="16" t="n">
+        <f aca="false">D13</f>
+        <v>14000</v>
+      </c>
+      <c r="E22" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
-        <v>510</v>
-      </c>
-      <c r="B22" s="31" t="n">
-        <f aca="false">SUM(B17:B21)</f>
+      <c r="F22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>514</v>
+      </c>
+      <c r="B23" s="31" t="n">
+        <f aca="false">SUM(B18:B22)</f>
+        <v>100825</v>
+      </c>
+      <c r="C23" s="31" t="n">
+        <f aca="false">SUM(C18:C22)</f>
         <v>116606.25</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="D23" s="31" t="n">
+        <f aca="false">SUM(D18:D22)</f>
+        <v>135843.75</v>
+      </c>
+      <c r="E23" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D22" s="2"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
-        <v>511</v>
-      </c>
-      <c r="B23" s="18" t="n">
-        <v>140000</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>442</v>
-      </c>
-      <c r="D23" s="2"/>
+      <c r="F23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>512</v>
-      </c>
-      <c r="B24" s="8" t="n">
-        <f aca="false">B23-B22</f>
+        <v>515</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="18" t="n">
+        <v>140000</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="F24" s="2"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>516</v>
+      </c>
+      <c r="B25" s="8" t="n">
+        <f aca="false">$C$24-B23</f>
+        <v>39175</v>
+      </c>
+      <c r="C25" s="8" t="n">
+        <f aca="false">$C$24-C23</f>
         <v>23393.75</v>
       </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
-        <v>513</v>
-      </c>
-      <c r="B25" s="37" t="n">
-        <f aca="false">B6*(B22/B5)*B14</f>
+      <c r="D25" s="8" t="n">
+        <f aca="false">$C$24-D23</f>
+        <v>4156.25</v>
+      </c>
+      <c r="E25" s="7"/>
+      <c r="F25" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>517</v>
+      </c>
+      <c r="B26" s="37" t="n">
+        <f aca="false">B6*(B23/B5)*B14</f>
+        <v>154.202941176471</v>
+      </c>
+      <c r="C26" s="37" t="n">
+        <f aca="false">C6*(C23/C5)*C14</f>
         <v>219.494117647059</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D26" s="37" t="n">
+        <f aca="false">D6*(D23/D5)*D14</f>
+        <v>303.650735294118</v>
+      </c>
+      <c r="E26" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D25" s="2"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-    </row>
-    <row r="27" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
-        <v>514</v>
-      </c>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
+      <c r="F26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+    </row>
+    <row r="28" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>518</v>
+      </c>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A27:D27"/>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A28:F28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Links: add contextual placements from relevant domains and on-site link assets alongside digital PR; split the budget line
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015LEzkrfcXznaX9ERkNGL27
</commit_message>
<xml_diff>
--- a/SEO_003_audit_and_refresh_model.xlsx
+++ b/SEO_003_audit_and_refresh_model.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1463" uniqueCount="764">
   <si>
     <t xml:space="preserve">SEO recovery plan: audit and refresh model</t>
   </si>
@@ -1195,13 +1195,13 @@
     <t xml:space="preserve">9-12</t>
   </si>
   <si>
-    <t xml:space="preserve">P3 refreshes (receipt scanning for citation, fraud statistics yearly update); internal links from the two strongest blog pages into the comparison hub; data study #1 scoped with product and legal</t>
+    <t xml:space="preserve">P3 refreshes (receipt scanning for citation, fraud statistics yearly update); internal links from the two strongest blog pages into the comparison hub; first batch of relevant-domain outreach aimed at the refreshed guides; data study #1 scoped with product and legal</t>
   </si>
   <si>
     <t xml:space="preserve">Content Manager, SEO Specialist</t>
   </si>
   <si>
-    <t xml:space="preserve">8 more refreshes live; internal link map; data study brief</t>
+    <t xml:space="preserve">8 more refreshes live; internal link map; outreach list with relevance notes; data study brief</t>
   </si>
   <si>
     <t xml:space="preserve">Legal sign-off on anonymized spend data</t>
@@ -1264,7 +1264,7 @@
     <t xml:space="preserve">Q2 (months 4 to 6)</t>
   </si>
   <si>
-    <t xml:space="preserve">Rules run on all 400 posts. 8 refreshes a month, consolidations by cluster. Data study #1 with outreach. Comparison hub: vs-ramp, vs-brex, 2 new comparison pages, 1 alternatives page. Template library with download-to-signup.</t>
+    <t xml:space="preserve">Rules run on all 400 posts. 8 refreshes a month, consolidations by cluster. Data study #1 with outreach. Contextual link placements from relevant domains running at 6 to 10 a month, aimed at the refreshed guides. Comparison hub: vs-ramp, vs-brex, 2 new comparison pages, 1 alternatives page. Template library with download-to-signup.</t>
   </si>
   <si>
     <t xml:space="preserve">Sprint 2: comparison page template (tables, schema, CTA components), template download flow, sitemap and removal handling.</t>
@@ -1417,7 +1417,13 @@
     <t xml:space="preserve">Digital PR and data study (freelancer retainer)</t>
   </si>
   <si>
-    <t xml:space="preserve">One original data asset a quarter from anonymized, aggregated product data plus outreach. No paid links at any price.</t>
+    <t xml:space="preserve">One original data asset a quarter from anonymized, aggregated product data, pitched to finance and business press. No paid links at any price.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contextual link outreach to relevant domains</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Editorial placements on finance, accounting, B2B software and business operations sites, pointing at the refreshed guides and comparison pages. Target 6 to 10 a month. No networks, no directories, no paid placements.</t>
   </si>
   <si>
     <t xml:space="preserve">WordPress speed and template contractor</t>
@@ -3142,7 +3148,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3152,7 +3158,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3170,22 +3176,22 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>344</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3193,19 +3199,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3213,19 +3219,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3233,19 +3239,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3253,19 +3259,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3273,19 +3279,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3293,19 +3299,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3313,19 +3319,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3333,19 +3339,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3353,19 +3359,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
   </sheetData>
@@ -3405,7 +3411,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3420,7 +3426,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3448,1533 +3454,1533 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>116</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H5" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H6" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="K6" s="19"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H7" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B8" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H8" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I8" s="19" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="I9" s="19" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="J9" s="19" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="I10" s="19" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="J10" s="19" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="K10" s="19"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H11" s="19" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="I11" s="19" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="I12" s="19" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="K12" s="19"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B13" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="I13" s="19" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="J13" s="19" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="K13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B14" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H14" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I14" s="19" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="J14" s="19" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="K14" s="19" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B15" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H15" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I15" s="19" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="J15" s="19" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="K15" s="19" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B16" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H16" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I16" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="K16" s="19" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H17" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I17" s="19" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="J17" s="19" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="K17" s="19" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B18" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H18" s="19" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="I18" s="19" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="J18" s="19" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="K18" s="19"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="I19" s="19" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="J19" s="19" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="K19" s="19"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B20" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H20" s="19" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="I20" s="19" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="J20" s="19" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="K20" s="19" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B21" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="I21" s="19" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="J21" s="19" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="K21" s="19"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B22" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H22" s="19" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="I22" s="19" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="J22" s="19" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="K22" s="19"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B23" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H23" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I23" s="19" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="J23" s="19" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="K23" s="19" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B24" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H24" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I24" s="19" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="J24" s="19" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="K24" s="19"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B25" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H25" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I25" s="19" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="J25" s="19" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="K25" s="19"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H26" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I26" s="19" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="J26" s="19" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="K26" s="19"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="I27" s="19" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="J27" s="19" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="K27" s="19"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="I28" s="19" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="J28" s="19" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="K28" s="19"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B29" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="I29" s="19" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="J29" s="19" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="K29" s="19" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="I30" s="19" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="J30" s="19" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="K30" s="19" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="I31" s="19" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="J31" s="19" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="K31" s="19" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B32" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H32" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I32" s="19" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="J32" s="19" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="K32" s="19" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B33" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F33" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H33" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I33" s="19" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="J33" s="19" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="K33" s="19"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B34" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H34" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I34" s="19" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="J34" s="19" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="K34" s="19"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B35" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H35" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I35" s="19" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="J35" s="19" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="K35" s="19"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B36" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="I36" s="19" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="J36" s="19" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="K36" s="19" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B37" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="I37" s="19" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="J37" s="19" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="K37" s="19"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B38" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G38" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="I38" s="19" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="J38" s="19" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="K38" s="19"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B39" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E39" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="I39" s="19" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="J39" s="19" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="K39" s="19"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B40" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="I40" s="19" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="J40" s="19" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="K40" s="19"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B41" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H41" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I41" s="19" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="J41" s="19" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="K41" s="19"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B42" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H42" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I42" s="19" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="J42" s="19" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="K42" s="19" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B43" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D43" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E43" s="19" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H43" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I43" s="19" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="J43" s="19" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="K43" s="19"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B44" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D44" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E44" s="19" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H44" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I44" s="19" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="J44" s="19" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="K44" s="19" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B45" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E45" s="19" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="I45" s="19" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="J45" s="19" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="K45" s="19" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B46" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D46" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="I46" s="19" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="J46" s="19" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="K46" s="19" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B47" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E47" s="19" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G47" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="I47" s="19" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="J47" s="19" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="K47" s="19" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B48" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D48" s="19" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F48" s="19" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G48" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="I48" s="19" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="J48" s="19" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="K48" s="19" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4992,7 +4998,7 @@
     </row>
     <row r="50" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B50" s="14"/>
       <c r="C50" s="14"/>
@@ -5020,7 +5026,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -5035,7 +5041,7 @@
     </row>
     <row r="53" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -5050,7 +5056,7 @@
     </row>
     <row r="54" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B54" s="14"/>
       <c r="C54" s="14"/>
@@ -5065,7 +5071,7 @@
     </row>
     <row r="55" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="B55" s="14"/>
       <c r="C55" s="14"/>
@@ -5080,7 +5086,7 @@
     </row>
     <row r="56" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
@@ -5095,7 +5101,7 @@
     </row>
     <row r="57" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
@@ -5110,7 +5116,7 @@
     </row>
     <row r="58" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B58" s="14"/>
       <c r="C58" s="14"/>
@@ -5165,7 +5171,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5184,7 +5190,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -5203,7 +5209,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -5222,66 +5228,66 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F5" s="20" t="n">
         <v>2026</v>
@@ -5316,19 +5322,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F6" s="20" t="n">
         <v>2026</v>
@@ -5363,19 +5369,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F7" s="20" t="n">
         <v>2026</v>
@@ -5410,19 +5416,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F8" s="20" t="n">
         <v>2026</v>
@@ -5457,19 +5463,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F9" s="20" t="n">
         <v>2026</v>
@@ -5504,19 +5510,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F10" s="20" t="n">
         <v>2026</v>
@@ -5551,7 +5557,7 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
@@ -5587,7 +5593,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -5606,40 +5612,40 @@
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
@@ -5647,19 +5653,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="F15" s="20" t="n">
         <v>8563</v>
@@ -5689,19 +5695,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="F16" s="20" t="n">
         <v>5382</v>
@@ -5731,19 +5737,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="F17" s="20" t="n">
         <v>4433</v>
@@ -5773,19 +5779,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="F18" s="20" t="n">
         <v>15000</v>
@@ -5815,19 +5821,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="F19" s="20" t="n">
         <v>6760</v>
@@ -5857,19 +5863,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="F20" s="20" t="n">
         <v>13667</v>
@@ -5899,19 +5905,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="F21" s="20" t="n">
         <v>31476</v>
@@ -5941,19 +5947,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="F22" s="20" t="n">
         <v>14045</v>
@@ -5983,19 +5989,19 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="F23" s="20" t="n">
         <v>36536</v>
@@ -6025,16 +6031,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E24" s="19" t="s">
         <v>111</v>
@@ -6067,19 +6073,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="F25" s="20" t="n">
         <v>47344</v>
@@ -6109,19 +6115,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="F26" s="20" t="n">
         <v>26473</v>
@@ -6151,19 +6157,19 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="F27" s="20" t="n">
         <v>14994</v>
@@ -6193,19 +6199,19 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="F28" s="20" t="n">
         <v>3225</v>
@@ -6235,19 +6241,19 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="F29" s="20" t="n">
         <v>4345</v>
@@ -6277,19 +6283,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>4418</v>
@@ -6319,19 +6325,19 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>6808</v>
@@ -6361,19 +6367,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>10232</v>
@@ -6403,19 +6409,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>11650</v>
@@ -6445,19 +6451,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>11323</v>
@@ -6487,19 +6493,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>18043</v>
@@ -6529,19 +6535,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>14414</v>
@@ -6571,16 +6577,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E37" s="19" t="s">
         <v>111</v>
@@ -6613,19 +6619,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>22928</v>
@@ -6655,19 +6661,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C39" s="19" t="s">
+        <v>746</v>
+      </c>
+      <c r="D39" s="19" t="s">
+        <v>747</v>
+      </c>
+      <c r="E39" s="19" t="s">
         <v>744</v>
-      </c>
-      <c r="D39" s="19" t="s">
-        <v>745</v>
-      </c>
-      <c r="E39" s="19" t="s">
-        <v>742</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>32985</v>
@@ -6697,19 +6703,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D40" s="19" t="s">
+        <v>747</v>
+      </c>
+      <c r="E40" s="19" t="s">
         <v>745</v>
-      </c>
-      <c r="E40" s="19" t="s">
-        <v>743</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>17453</v>
@@ -6756,7 +6762,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -6775,25 +6781,25 @@
     </row>
     <row r="43" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
@@ -6806,7 +6812,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="B44" s="16" t="n">
         <f aca="false">SUM(J15:J26)</f>
@@ -6843,7 +6849,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="B45" s="16" t="n">
         <f aca="false">SUM(J28:J39)</f>
@@ -6880,7 +6886,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="17" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -6916,7 +6922,7 @@
     </row>
     <row r="48" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="B48" s="14"/>
       <c r="C48" s="14"/>
@@ -6965,7 +6971,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6973,7 +6979,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -6987,16 +6993,16 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>403</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7007,10 +7013,10 @@
         <v>0.398</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7021,7 +7027,7 @@
         <v>0.187</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D6" s="10"/>
     </row>
@@ -7033,7 +7039,7 @@
         <v>0.102</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D7" s="10"/>
     </row>
@@ -7045,7 +7051,7 @@
         <v>0.072</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D8" s="10"/>
     </row>
@@ -7057,7 +7063,7 @@
         <v>0.051</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D9" s="10"/>
     </row>
@@ -7069,7 +7075,7 @@
         <v>0.044</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D10" s="10"/>
     </row>
@@ -7081,7 +7087,7 @@
         <v>0.03</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D11" s="10"/>
     </row>
@@ -7093,7 +7099,7 @@
         <v>0.021</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D12" s="10"/>
     </row>
@@ -7105,7 +7111,7 @@
         <v>0.019</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D13" s="10"/>
     </row>
@@ -7117,7 +7123,7 @@
         <v>0.016</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D14" s="10"/>
     </row>
@@ -7132,7 +7138,7 @@
         <v>454</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11683,7 +11689,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
@@ -11777,7 +11783,7 @@
         <v>460</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>454</v>
@@ -11791,7 +11797,7 @@
         <v>462</v>
       </c>
       <c r="B9" s="33" t="n">
-        <v>2500</v>
+        <v>1500</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>454</v>
@@ -11805,7 +11811,7 @@
         <v>464</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>1500</v>
+        <v>2500</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>454</v>
@@ -11819,7 +11825,7 @@
         <v>466</v>
       </c>
       <c r="B11" s="33" t="n">
-        <v>700</v>
+        <v>1500</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>454</v>
@@ -11833,7 +11839,7 @@
         <v>468</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>2500</v>
+        <v>700</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>454</v>
@@ -11842,112 +11848,126 @@
         <v>469</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>470</v>
       </c>
-      <c r="B13" s="34" t="n">
-        <f aca="false">SUM(B5:B12)</f>
-        <v>15000</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="B13" s="33" t="n">
+        <v>2500</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>471</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>471</v>
-      </c>
-      <c r="B14" s="33" t="n">
+        <v>472</v>
+      </c>
+      <c r="B14" s="34" t="n">
+        <f aca="false">SUM(B5:B13)</f>
         <v>15000</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>442</v>
-      </c>
+      <c r="C14" s="2"/>
       <c r="D14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>472</v>
-      </c>
-      <c r="B15" s="35" t="n">
-        <f aca="false">B14-B13</f>
+        <v>473</v>
+      </c>
+      <c r="B15" s="33" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>474</v>
+      </c>
+      <c r="B16" s="35" t="n">
+        <f aca="false">B15-B14</f>
         <v>0</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>473</v>
-      </c>
+      <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>474</v>
-      </c>
-      <c r="B18" s="7" t="n">
+      <c r="A18" s="11" t="s">
+        <v>475</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>476</v>
+      </c>
+      <c r="B19" s="7" t="n">
         <f aca="false">4*12</f>
         <v>48</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>475</v>
-      </c>
-      <c r="B19" s="7" t="n">
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="B20" s="7" t="n">
         <f aca="false">8*12</f>
         <v>96</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>476</v>
-      </c>
-      <c r="B20" s="17" t="n">
-        <v>80</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>408</v>
-      </c>
+      <c r="C20" s="2"/>
       <c r="D20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>477</v>
-      </c>
-      <c r="B21" s="7" t="n">
-        <f aca="false">B18+B19+B20</f>
+        <v>478</v>
+      </c>
+      <c r="B21" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>479</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <f aca="false">B19+B20+B21</f>
         <v>224</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>478</v>
-      </c>
-      <c r="B22" s="7" t="n">
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="s">
+        <v>480</v>
+      </c>
+      <c r="B23" s="7" t="n">
         <f aca="false">50*2</f>
         <v>100</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C23" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="D22" s="10" t="s">
-        <v>479</v>
+      <c r="D23" s="10" t="s">
+        <v>481</v>
       </c>
     </row>
   </sheetData>
@@ -11980,7 +12000,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -11990,7 +12010,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -12000,7 +12020,7 @@
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
@@ -12010,27 +12030,27 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>403</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>85000</v>
@@ -12045,12 +12065,12 @@
         <v>442</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>100</v>
@@ -12065,12 +12085,12 @@
         <v>454</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>20000</v>
@@ -12085,12 +12105,12 @@
         <v>454</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B8" s="36" t="n">
         <v>0.25</v>
@@ -12105,12 +12125,12 @@
         <v>408</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B9" s="36" t="n">
         <v>0.15</v>
@@ -12125,12 +12145,12 @@
         <v>454</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B10" s="36" t="n">
         <v>0.4</v>
@@ -12145,12 +12165,12 @@
         <v>408</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B11" s="36" t="n">
         <v>0.25</v>
@@ -12165,12 +12185,12 @@
         <v>408</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>2000</v>
@@ -12185,12 +12205,12 @@
         <v>408</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B13" s="18" t="n">
         <v>5000</v>
@@ -12205,12 +12225,12 @@
         <v>408</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B14" s="36" t="n">
         <v>1.3</v>
@@ -12225,7 +12245,7 @@
         <v>408</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12238,7 +12258,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -12249,13 +12269,13 @@
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6"/>
       <c r="B17" s="6" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>403</v>
@@ -12264,7 +12284,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B18" s="16" t="n">
         <f aca="false">B5</f>
@@ -12285,7 +12305,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B19" s="16" t="n">
         <f aca="false">B7*B8</f>
@@ -12306,7 +12326,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B20" s="16" t="n">
         <f aca="false">B5*(1-B11)*B10*B9</f>
@@ -12327,7 +12347,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B21" s="16" t="n">
         <f aca="false">B12</f>
@@ -12348,7 +12368,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B22" s="16" t="n">
         <f aca="false">B13</f>
@@ -12369,7 +12389,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B23" s="31" t="n">
         <f aca="false">SUM(B18:B22)</f>
@@ -12390,7 +12410,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="18" t="n">
@@ -12404,7 +12424,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">$C$24-B23</f>
@@ -12423,7 +12443,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B26" s="37" t="n">
         <f aca="false">B6*(B23/B5)*B14</f>
@@ -12452,7 +12472,7 @@
     </row>
     <row r="28" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>

</xml_diff>

<commit_message>
Use the brief's tools explicitly: Clearscope in the refresh workflow, reverse-silo internal linking, named link targets, reserve purpose stated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015LEzkrfcXznaX9ERkNGL27
</commit_message>
<xml_diff>
--- a/SEO_003_audit_and_refresh_model.xlsx
+++ b/SEO_003_audit_and_refresh_model.xlsx
@@ -1138,13 +1138,13 @@
     <t xml:space="preserve">3-5</t>
   </si>
   <si>
-    <t xml:space="preserve">what-is-expense-management refreshed for depth and AI Overview citation; cannibal merged and redirected</t>
+    <t xml:space="preserve">what-is-expense-management refreshed for depth and AI Overview citation, brief built in Clearscope against the current top 10; cannibal merged and redirected</t>
   </si>
   <si>
     <t xml:space="preserve">Content Manager, freelancer</t>
   </si>
   <si>
-    <t xml:space="preserve">Refreshed URL live; Search Console URL filter saved for the holdout</t>
+    <t xml:space="preserve">Refreshed URL live; Clearscope score on the new draft; Search Console URL filter saved for the holdout</t>
   </si>
   <si>
     <t xml:space="preserve">Redirect map</t>
@@ -1279,7 +1279,7 @@
     <t xml:space="preserve">Refresh pipeline at full pace. Data study #2. First hire decision (content strategist or editor) once the 6-month freeze ends, only if refresh throughput is the bottleneck. Spend management cluster complete.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 3: internal linking automation from the strongest pages to the comparison and product pages, hub pages.</t>
+    <t xml:space="preserve">Sprint 3: internal linking automation built as a reverse silo (guides up to topic hubs, hubs to the comparison and product pages, every link reciprocated), hub pages.</t>
   </si>
   <si>
     <t xml:space="preserve">250+ posts actioned. Organic conversions about +80%. Traffic 110K to 120K.</t>

</xml_diff>

<commit_message>
Option B content model (client voice skill, AI drafting, editor as validation layer, saving to links); PDF back to 4 pages
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015LEzkrfcXznaX9ERkNGL27
</commit_message>
<xml_diff>
--- a/SEO_003_audit_and_refresh_model.xlsx
+++ b/SEO_003_audit_and_refresh_model.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1463" uniqueCount="764">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1486" uniqueCount="778">
   <si>
     <t xml:space="preserve">SEO recovery plan: audit and refresh model</t>
   </si>
@@ -1478,6 +1478,48 @@
   </si>
   <si>
     <t xml:space="preserve">50 posts in 6 months in the brief. We cannot match it on new posts (48 a year). Refreshes and consolidations are where our effort goes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option B: AI drafting in the client's voice, editor as the validation layer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A dedicated Claude project with a voice skill built from interviews with the Content Manager and two subject experts (tone, style, how they talk to customers). Drafts come from Clearscope briefs; a freelance editor checks facts, sources, voice and CTA on every piece before it publishes. The saving moves to contextual link outreach. Testable in Q2: run it on half the refreshes and compare with freelancer-written pages against the holdout.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freelance model: content cost (new posts plus refreshes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From the lines above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option B: editor review, 12 pieces x $75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freelance editor, one pass per piece: facts, sources, voice, CTA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option B: AI tooling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claude subscription and the voice-skill project.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option B: monthly content cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly saving moved to contextual link outreach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contextual link outreach under Option B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 to 20 qualified placements a month at this level.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-off setup: interviews and the voice skill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid from the reserve in month one.</t>
   </si>
   <si>
     <t xml:space="preserve">Month-12 targets: three scenarios</t>
@@ -2508,7 +2550,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2650,6 +2692,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3148,7 +3194,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>521</v>
+        <v>535</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3158,7 +3204,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>522</v>
+        <v>536</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3176,22 +3222,22 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>523</v>
+        <v>537</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>524</v>
+        <v>538</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>525</v>
+        <v>539</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>344</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>526</v>
+        <v>540</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>527</v>
+        <v>541</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3199,19 +3245,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>528</v>
+        <v>542</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>529</v>
+        <v>543</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>530</v>
+        <v>544</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>531</v>
+        <v>545</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3219,19 +3265,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>532</v>
+        <v>546</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>533</v>
+        <v>547</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>534</v>
+        <v>548</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>535</v>
+        <v>549</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3239,19 +3285,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>536</v>
+        <v>550</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>537</v>
+        <v>551</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>538</v>
+        <v>552</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>539</v>
+        <v>553</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>540</v>
+        <v>554</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3259,19 +3305,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>541</v>
+        <v>555</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>542</v>
+        <v>556</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>543</v>
+        <v>557</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>544</v>
+        <v>558</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3279,19 +3325,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>545</v>
+        <v>559</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>546</v>
+        <v>560</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>547</v>
+        <v>561</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>548</v>
+        <v>562</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>549</v>
+        <v>563</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3299,19 +3345,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>550</v>
+        <v>564</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>551</v>
+        <v>565</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>552</v>
+        <v>566</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>553</v>
+        <v>567</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3319,19 +3365,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>554</v>
+        <v>568</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>555</v>
+        <v>569</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>556</v>
+        <v>570</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>557</v>
+        <v>571</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>558</v>
+        <v>572</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3339,19 +3385,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>559</v>
+        <v>573</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>560</v>
+        <v>574</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>354</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>561</v>
+        <v>575</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>562</v>
+        <v>576</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3359,19 +3405,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>563</v>
+        <v>577</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>564</v>
+        <v>578</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>564</v>
+        <v>578</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>565</v>
+        <v>579</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>566</v>
+        <v>580</v>
       </c>
     </row>
   </sheetData>
@@ -3411,7 +3457,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>567</v>
+        <v>581</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3426,7 +3472,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>568</v>
+        <v>582</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3454,1533 +3500,1533 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>569</v>
+        <v>583</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>570</v>
+        <v>584</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>571</v>
+        <v>585</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>572</v>
+        <v>586</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>573</v>
+        <v>587</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>574</v>
+        <v>588</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>575</v>
+        <v>589</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>576</v>
+        <v>590</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>116</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H5" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>585</v>
+        <v>599</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>586</v>
+        <v>600</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>587</v>
+        <v>601</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H6" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>588</v>
+        <v>602</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>589</v>
+        <v>603</v>
       </c>
       <c r="K6" s="19"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H7" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>591</v>
+        <v>605</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>592</v>
+        <v>606</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B8" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H8" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I8" s="19" t="s">
-        <v>593</v>
+        <v>607</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>594</v>
+        <v>608</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>595</v>
+        <v>609</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H9" s="19" t="s">
-        <v>596</v>
+        <v>610</v>
       </c>
       <c r="I9" s="19" t="s">
-        <v>597</v>
+        <v>611</v>
       </c>
       <c r="J9" s="19" t="s">
-        <v>598</v>
+        <v>612</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>599</v>
+        <v>613</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H10" s="19" t="s">
-        <v>600</v>
+        <v>614</v>
       </c>
       <c r="I10" s="19" t="s">
-        <v>601</v>
+        <v>615</v>
       </c>
       <c r="J10" s="19" t="s">
-        <v>602</v>
+        <v>616</v>
       </c>
       <c r="K10" s="19"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H11" s="19" t="s">
-        <v>603</v>
+        <v>617</v>
       </c>
       <c r="I11" s="19" t="s">
-        <v>604</v>
+        <v>618</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>605</v>
+        <v>619</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>606</v>
+        <v>620</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H12" s="19" t="s">
-        <v>607</v>
+        <v>621</v>
       </c>
       <c r="I12" s="19" t="s">
-        <v>608</v>
+        <v>622</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>609</v>
+        <v>623</v>
       </c>
       <c r="K12" s="19"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B13" s="19" t="s">
         <v>142</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H13" s="19" t="s">
-        <v>610</v>
+        <v>624</v>
       </c>
       <c r="I13" s="19" t="s">
-        <v>611</v>
+        <v>625</v>
       </c>
       <c r="J13" s="19" t="s">
-        <v>612</v>
+        <v>626</v>
       </c>
       <c r="K13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B14" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H14" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I14" s="19" t="s">
-        <v>614</v>
+        <v>628</v>
       </c>
       <c r="J14" s="19" t="s">
-        <v>615</v>
+        <v>629</v>
       </c>
       <c r="K14" s="19" t="s">
-        <v>616</v>
+        <v>630</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B15" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H15" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I15" s="19" t="s">
-        <v>585</v>
+        <v>599</v>
       </c>
       <c r="J15" s="19" t="s">
-        <v>617</v>
+        <v>631</v>
       </c>
       <c r="K15" s="19" t="s">
-        <v>618</v>
+        <v>632</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B16" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H16" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I16" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>619</v>
+        <v>633</v>
       </c>
       <c r="K16" s="19" t="s">
-        <v>620</v>
+        <v>634</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H17" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I17" s="19" t="s">
-        <v>621</v>
+        <v>635</v>
       </c>
       <c r="J17" s="19" t="s">
-        <v>622</v>
+        <v>636</v>
       </c>
       <c r="K17" s="19" t="s">
-        <v>623</v>
+        <v>637</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B18" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H18" s="19" t="s">
-        <v>596</v>
+        <v>610</v>
       </c>
       <c r="I18" s="19" t="s">
-        <v>624</v>
+        <v>638</v>
       </c>
       <c r="J18" s="19" t="s">
-        <v>625</v>
+        <v>639</v>
       </c>
       <c r="K18" s="19"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>600</v>
+        <v>614</v>
       </c>
       <c r="I19" s="19" t="s">
-        <v>626</v>
+        <v>640</v>
       </c>
       <c r="J19" s="19" t="s">
-        <v>627</v>
+        <v>641</v>
       </c>
       <c r="K19" s="19"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B20" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H20" s="19" t="s">
-        <v>603</v>
+        <v>617</v>
       </c>
       <c r="I20" s="19" t="s">
-        <v>628</v>
+        <v>642</v>
       </c>
       <c r="J20" s="19" t="s">
-        <v>629</v>
+        <v>643</v>
       </c>
       <c r="K20" s="19" t="s">
-        <v>630</v>
+        <v>644</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B21" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H21" s="19" t="s">
-        <v>607</v>
+        <v>621</v>
       </c>
       <c r="I21" s="19" t="s">
-        <v>631</v>
+        <v>645</v>
       </c>
       <c r="J21" s="19" t="s">
-        <v>632</v>
+        <v>646</v>
       </c>
       <c r="K21" s="19"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B22" s="19" t="s">
         <v>163</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H22" s="19" t="s">
-        <v>610</v>
+        <v>624</v>
       </c>
       <c r="I22" s="19" t="s">
-        <v>633</v>
+        <v>647</v>
       </c>
       <c r="J22" s="19" t="s">
-        <v>634</v>
+        <v>648</v>
       </c>
       <c r="K22" s="19"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B23" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H23" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I23" s="19" t="s">
-        <v>636</v>
+        <v>650</v>
       </c>
       <c r="J23" s="19" t="s">
-        <v>637</v>
+        <v>651</v>
       </c>
       <c r="K23" s="19" t="s">
-        <v>638</v>
+        <v>652</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B24" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H24" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I24" s="19" t="s">
-        <v>639</v>
+        <v>653</v>
       </c>
       <c r="J24" s="19" t="s">
-        <v>640</v>
+        <v>654</v>
       </c>
       <c r="K24" s="19"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B25" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H25" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I25" s="19" t="s">
-        <v>641</v>
+        <v>655</v>
       </c>
       <c r="J25" s="19" t="s">
-        <v>642</v>
+        <v>656</v>
       </c>
       <c r="K25" s="19"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B26" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H26" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I26" s="19" t="s">
-        <v>643</v>
+        <v>657</v>
       </c>
       <c r="J26" s="19" t="s">
-        <v>644</v>
+        <v>658</v>
       </c>
       <c r="K26" s="19"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B27" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>596</v>
+        <v>610</v>
       </c>
       <c r="I27" s="19" t="s">
-        <v>645</v>
+        <v>659</v>
       </c>
       <c r="J27" s="19" t="s">
-        <v>646</v>
+        <v>660</v>
       </c>
       <c r="K27" s="19"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B28" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H28" s="19" t="s">
-        <v>600</v>
+        <v>614</v>
       </c>
       <c r="I28" s="19" t="s">
-        <v>647</v>
+        <v>661</v>
       </c>
       <c r="J28" s="19" t="s">
-        <v>648</v>
+        <v>662</v>
       </c>
       <c r="K28" s="19"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B29" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>603</v>
+        <v>617</v>
       </c>
       <c r="I29" s="19" t="s">
-        <v>649</v>
+        <v>663</v>
       </c>
       <c r="J29" s="19" t="s">
-        <v>650</v>
+        <v>664</v>
       </c>
       <c r="K29" s="19" t="s">
-        <v>651</v>
+        <v>665</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B30" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H30" s="19" t="s">
-        <v>607</v>
+        <v>621</v>
       </c>
       <c r="I30" s="19" t="s">
-        <v>631</v>
+        <v>645</v>
       </c>
       <c r="J30" s="19" t="s">
-        <v>652</v>
+        <v>666</v>
       </c>
       <c r="K30" s="19" t="s">
-        <v>653</v>
+        <v>667</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B31" s="19" t="s">
         <v>170</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>635</v>
+        <v>649</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H31" s="19" t="s">
-        <v>610</v>
+        <v>624</v>
       </c>
       <c r="I31" s="19" t="s">
-        <v>654</v>
+        <v>668</v>
       </c>
       <c r="J31" s="19" t="s">
-        <v>655</v>
+        <v>669</v>
       </c>
       <c r="K31" s="19" t="s">
-        <v>656</v>
+        <v>670</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B32" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>658</v>
+        <v>672</v>
       </c>
       <c r="H32" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I32" s="19" t="s">
-        <v>659</v>
+        <v>673</v>
       </c>
       <c r="J32" s="19" t="s">
-        <v>660</v>
+        <v>674</v>
       </c>
       <c r="K32" s="19" t="s">
-        <v>661</v>
+        <v>675</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B33" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="F33" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>658</v>
+        <v>672</v>
       </c>
       <c r="H33" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I33" s="19" t="s">
-        <v>662</v>
+        <v>676</v>
       </c>
       <c r="J33" s="19" t="s">
-        <v>663</v>
+        <v>677</v>
       </c>
       <c r="K33" s="19"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B34" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>658</v>
+        <v>672</v>
       </c>
       <c r="H34" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I34" s="19" t="s">
-        <v>664</v>
+        <v>678</v>
       </c>
       <c r="J34" s="19" t="s">
-        <v>665</v>
+        <v>679</v>
       </c>
       <c r="K34" s="19"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B35" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>658</v>
+        <v>672</v>
       </c>
       <c r="H35" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I35" s="19" t="s">
-        <v>666</v>
+        <v>680</v>
       </c>
       <c r="J35" s="19" t="s">
-        <v>667</v>
+        <v>681</v>
       </c>
       <c r="K35" s="19"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B36" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>658</v>
+        <v>672</v>
       </c>
       <c r="H36" s="19" t="s">
-        <v>596</v>
+        <v>610</v>
       </c>
       <c r="I36" s="19" t="s">
-        <v>659</v>
+        <v>673</v>
       </c>
       <c r="J36" s="19" t="s">
-        <v>668</v>
+        <v>682</v>
       </c>
       <c r="K36" s="19" t="s">
-        <v>669</v>
+        <v>683</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B37" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E37" s="19" t="s">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>658</v>
+        <v>672</v>
       </c>
       <c r="H37" s="19" t="s">
-        <v>600</v>
+        <v>614</v>
       </c>
       <c r="I37" s="19" t="s">
-        <v>670</v>
+        <v>684</v>
       </c>
       <c r="J37" s="19" t="s">
-        <v>671</v>
+        <v>685</v>
       </c>
       <c r="K37" s="19"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B38" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G38" s="19" t="s">
-        <v>658</v>
+        <v>672</v>
       </c>
       <c r="H38" s="19" t="s">
-        <v>603</v>
+        <v>617</v>
       </c>
       <c r="I38" s="19" t="s">
-        <v>672</v>
+        <v>686</v>
       </c>
       <c r="J38" s="19" t="s">
-        <v>673</v>
+        <v>687</v>
       </c>
       <c r="K38" s="19"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B39" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E39" s="19" t="s">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>658</v>
+        <v>672</v>
       </c>
       <c r="H39" s="19" t="s">
-        <v>607</v>
+        <v>621</v>
       </c>
       <c r="I39" s="19" t="s">
-        <v>674</v>
+        <v>688</v>
       </c>
       <c r="J39" s="19" t="s">
-        <v>675</v>
+        <v>689</v>
       </c>
       <c r="K39" s="19"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B40" s="19" t="s">
         <v>188</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>658</v>
+        <v>672</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>610</v>
+        <v>624</v>
       </c>
       <c r="I40" s="19" t="s">
-        <v>676</v>
+        <v>690</v>
       </c>
       <c r="J40" s="19" t="s">
-        <v>677</v>
+        <v>691</v>
       </c>
       <c r="K40" s="19"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B41" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>678</v>
+        <v>692</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H41" s="19" t="s">
         <v>347</v>
       </c>
       <c r="I41" s="19" t="s">
-        <v>611</v>
+        <v>625</v>
       </c>
       <c r="J41" s="19" t="s">
-        <v>679</v>
+        <v>693</v>
       </c>
       <c r="K41" s="19"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B42" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>678</v>
+        <v>692</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H42" s="19" t="s">
         <v>352</v>
       </c>
       <c r="I42" s="19" t="s">
-        <v>680</v>
+        <v>694</v>
       </c>
       <c r="J42" s="19" t="s">
-        <v>681</v>
+        <v>695</v>
       </c>
       <c r="K42" s="19" t="s">
-        <v>682</v>
+        <v>696</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B43" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D43" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E43" s="19" t="s">
-        <v>678</v>
+        <v>692</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H43" s="19" t="s">
         <v>357</v>
       </c>
       <c r="I43" s="19" t="s">
-        <v>641</v>
+        <v>655</v>
       </c>
       <c r="J43" s="19" t="s">
-        <v>683</v>
+        <v>697</v>
       </c>
       <c r="K43" s="19"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B44" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D44" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E44" s="19" t="s">
-        <v>678</v>
+        <v>692</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H44" s="19" t="s">
         <v>372</v>
       </c>
       <c r="I44" s="19" t="s">
-        <v>684</v>
+        <v>698</v>
       </c>
       <c r="J44" s="19" t="s">
-        <v>685</v>
+        <v>699</v>
       </c>
       <c r="K44" s="19" t="s">
-        <v>686</v>
+        <v>700</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B45" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E45" s="19" t="s">
-        <v>678</v>
+        <v>692</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>596</v>
+        <v>610</v>
       </c>
       <c r="I45" s="19" t="s">
-        <v>687</v>
+        <v>701</v>
       </c>
       <c r="J45" s="19" t="s">
-        <v>688</v>
+        <v>702</v>
       </c>
       <c r="K45" s="19" t="s">
-        <v>689</v>
+        <v>703</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B46" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D46" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>678</v>
+        <v>692</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H46" s="19" t="s">
-        <v>600</v>
+        <v>614</v>
       </c>
       <c r="I46" s="19" t="s">
-        <v>690</v>
+        <v>704</v>
       </c>
       <c r="J46" s="19" t="s">
-        <v>691</v>
+        <v>705</v>
       </c>
       <c r="K46" s="19" t="s">
-        <v>692</v>
+        <v>706</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B47" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E47" s="19" t="s">
-        <v>678</v>
+        <v>692</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G47" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H47" s="19" t="s">
-        <v>603</v>
+        <v>617</v>
       </c>
       <c r="I47" s="19" t="s">
-        <v>693</v>
+        <v>707</v>
       </c>
       <c r="J47" s="19" t="s">
-        <v>694</v>
+        <v>708</v>
       </c>
       <c r="K47" s="19" t="s">
-        <v>695</v>
+        <v>709</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B48" s="19" t="s">
         <v>243</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D48" s="19" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>678</v>
+        <v>692</v>
       </c>
       <c r="F48" s="19" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G48" s="19" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
       <c r="H48" s="19" t="s">
-        <v>607</v>
+        <v>621</v>
       </c>
       <c r="I48" s="19" t="s">
-        <v>696</v>
+        <v>710</v>
       </c>
       <c r="J48" s="19" t="s">
-        <v>697</v>
+        <v>711</v>
       </c>
       <c r="K48" s="19" t="s">
-        <v>698</v>
+        <v>712</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4998,7 +5044,7 @@
     </row>
     <row r="50" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="s">
-        <v>699</v>
+        <v>713</v>
       </c>
       <c r="B50" s="14"/>
       <c r="C50" s="14"/>
@@ -5026,7 +5072,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="s">
-        <v>700</v>
+        <v>714</v>
       </c>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -5041,7 +5087,7 @@
     </row>
     <row r="53" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="s">
-        <v>701</v>
+        <v>715</v>
       </c>
       <c r="B53" s="14"/>
       <c r="C53" s="14"/>
@@ -5056,7 +5102,7 @@
     </row>
     <row r="54" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>702</v>
+        <v>716</v>
       </c>
       <c r="B54" s="14"/>
       <c r="C54" s="14"/>
@@ -5071,7 +5117,7 @@
     </row>
     <row r="55" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="s">
-        <v>703</v>
+        <v>717</v>
       </c>
       <c r="B55" s="14"/>
       <c r="C55" s="14"/>
@@ -5086,7 +5132,7 @@
     </row>
     <row r="56" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="s">
-        <v>704</v>
+        <v>718</v>
       </c>
       <c r="B56" s="14"/>
       <c r="C56" s="14"/>
@@ -5101,7 +5147,7 @@
     </row>
     <row r="57" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="s">
-        <v>705</v>
+        <v>719</v>
       </c>
       <c r="B57" s="14"/>
       <c r="C57" s="14"/>
@@ -5116,7 +5162,7 @@
     </row>
     <row r="58" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="s">
-        <v>706</v>
+        <v>720</v>
       </c>
       <c r="B58" s="14"/>
       <c r="C58" s="14"/>
@@ -5171,7 +5217,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>707</v>
+        <v>721</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5190,7 +5236,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>708</v>
+        <v>722</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -5209,7 +5255,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>709</v>
+        <v>723</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -5228,66 +5274,66 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>569</v>
+        <v>583</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>525</v>
+        <v>539</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>710</v>
+        <v>724</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>571</v>
+        <v>585</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>711</v>
+        <v>725</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>712</v>
+        <v>726</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>713</v>
+        <v>727</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>714</v>
+        <v>728</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>715</v>
+        <v>729</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>716</v>
+        <v>730</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>717</v>
+        <v>731</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>718</v>
+        <v>732</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>719</v>
+        <v>733</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>720</v>
+        <v>734</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>721</v>
+        <v>735</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>722</v>
+        <v>736</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="F5" s="20" t="n">
         <v>2026</v>
@@ -5322,19 +5368,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>721</v>
+        <v>735</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>722</v>
+        <v>736</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="F6" s="20" t="n">
         <v>2026</v>
@@ -5369,19 +5415,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>721</v>
+        <v>735</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>722</v>
+        <v>736</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="F7" s="20" t="n">
         <v>2026</v>
@@ -5416,19 +5462,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>721</v>
+        <v>735</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>722</v>
+        <v>736</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="F8" s="20" t="n">
         <v>2026</v>
@@ -5463,19 +5509,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>721</v>
+        <v>735</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>722</v>
+        <v>736</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="F9" s="20" t="n">
         <v>2026</v>
@@ -5510,19 +5556,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>721</v>
+        <v>735</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>722</v>
+        <v>736</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="F10" s="20" t="n">
         <v>2026</v>
@@ -5557,7 +5603,7 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>723</v>
+        <v>737</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
@@ -5593,7 +5639,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>724</v>
+        <v>738</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -5612,40 +5658,40 @@
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>569</v>
+        <v>583</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>525</v>
+        <v>539</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>710</v>
+        <v>724</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>712</v>
+        <v>726</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>725</v>
+        <v>739</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>726</v>
+        <v>740</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>727</v>
+        <v>741</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>728</v>
+        <v>742</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>729</v>
+        <v>743</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>730</v>
+        <v>744</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>731</v>
+        <v>745</v>
       </c>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
@@ -5653,19 +5699,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E15" s="19" t="s">
-        <v>734</v>
+        <v>748</v>
       </c>
       <c r="F15" s="20" t="n">
         <v>8563</v>
@@ -5695,19 +5741,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>735</v>
+        <v>749</v>
       </c>
       <c r="F16" s="20" t="n">
         <v>5382</v>
@@ -5737,19 +5783,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>736</v>
+        <v>750</v>
       </c>
       <c r="F17" s="20" t="n">
         <v>4433</v>
@@ -5779,19 +5825,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>737</v>
+        <v>751</v>
       </c>
       <c r="F18" s="20" t="n">
         <v>15000</v>
@@ -5821,19 +5867,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>738</v>
+        <v>752</v>
       </c>
       <c r="F19" s="20" t="n">
         <v>6760</v>
@@ -5863,19 +5909,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>739</v>
+        <v>753</v>
       </c>
       <c r="F20" s="20" t="n">
         <v>13667</v>
@@ -5905,19 +5951,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>740</v>
+        <v>754</v>
       </c>
       <c r="F21" s="20" t="n">
         <v>31476</v>
@@ -5947,19 +5993,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>741</v>
+        <v>755</v>
       </c>
       <c r="F22" s="20" t="n">
         <v>14045</v>
@@ -5989,19 +6035,19 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>742</v>
+        <v>756</v>
       </c>
       <c r="F23" s="20" t="n">
         <v>36536</v>
@@ -6031,16 +6077,16 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E24" s="19" t="s">
         <v>111</v>
@@ -6073,19 +6119,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>743</v>
+        <v>757</v>
       </c>
       <c r="F25" s="20" t="n">
         <v>47344</v>
@@ -6115,19 +6161,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>744</v>
+        <v>758</v>
       </c>
       <c r="F26" s="20" t="n">
         <v>26473</v>
@@ -6157,19 +6203,19 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>745</v>
+        <v>759</v>
       </c>
       <c r="F27" s="20" t="n">
         <v>14994</v>
@@ -6199,19 +6245,19 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>734</v>
+        <v>748</v>
       </c>
       <c r="F28" s="20" t="n">
         <v>3225</v>
@@ -6241,19 +6287,19 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>735</v>
+        <v>749</v>
       </c>
       <c r="F29" s="20" t="n">
         <v>4345</v>
@@ -6283,19 +6329,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>736</v>
+        <v>750</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>4418</v>
@@ -6325,19 +6371,19 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>737</v>
+        <v>751</v>
       </c>
       <c r="F31" s="20" t="n">
         <v>6808</v>
@@ -6367,19 +6413,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>738</v>
+        <v>752</v>
       </c>
       <c r="F32" s="20" t="n">
         <v>10232</v>
@@ -6409,19 +6455,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>739</v>
+        <v>753</v>
       </c>
       <c r="F33" s="20" t="n">
         <v>11650</v>
@@ -6451,19 +6497,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>740</v>
+        <v>754</v>
       </c>
       <c r="F34" s="20" t="n">
         <v>11323</v>
@@ -6493,19 +6539,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>741</v>
+        <v>755</v>
       </c>
       <c r="F35" s="20" t="n">
         <v>18043</v>
@@ -6535,19 +6581,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>742</v>
+        <v>756</v>
       </c>
       <c r="F36" s="20" t="n">
         <v>14414</v>
@@ -6577,16 +6623,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E37" s="19" t="s">
         <v>111</v>
@@ -6619,19 +6665,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>743</v>
+        <v>757</v>
       </c>
       <c r="F38" s="20" t="n">
         <v>22928</v>
@@ -6661,19 +6707,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E39" s="19" t="s">
-        <v>744</v>
+        <v>758</v>
       </c>
       <c r="F39" s="20" t="n">
         <v>32985</v>
@@ -6703,19 +6749,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="19" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>732</v>
+        <v>746</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>746</v>
+        <v>760</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>745</v>
+        <v>759</v>
       </c>
       <c r="F40" s="20" t="n">
         <v>17453</v>
@@ -6762,7 +6808,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>748</v>
+        <v>762</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -6781,25 +6827,25 @@
     </row>
     <row r="43" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>749</v>
+        <v>763</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>750</v>
+        <v>764</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>751</v>
+        <v>765</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>752</v>
+        <v>766</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>753</v>
+        <v>767</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>754</v>
+        <v>768</v>
       </c>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
@@ -6812,7 +6858,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="B44" s="16" t="n">
         <f aca="false">SUM(J15:J26)</f>
@@ -6849,7 +6895,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>747</v>
+        <v>761</v>
       </c>
       <c r="B45" s="16" t="n">
         <f aca="false">SUM(J28:J39)</f>
@@ -6886,7 +6932,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="17" t="s">
-        <v>755</v>
+        <v>769</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -6922,7 +6968,7 @@
     </row>
     <row r="48" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
-        <v>756</v>
+        <v>770</v>
       </c>
       <c r="B48" s="14"/>
       <c r="C48" s="14"/>
@@ -6971,7 +7017,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>757</v>
+        <v>771</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6979,7 +7025,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>758</v>
+        <v>772</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -6993,41 +7039,41 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>759</v>
+        <v>773</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>760</v>
+        <v>774</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>403</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>525</v>
+        <v>539</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="38" t="n">
+      <c r="B5" s="39" t="n">
         <v>0.398</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>762</v>
+        <v>776</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="38" t="n">
+      <c r="B6" s="39" t="n">
         <v>0.187</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D6" s="10"/>
     </row>
@@ -7035,11 +7081,11 @@
       <c r="A7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="39" t="n">
         <v>0.102</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D7" s="10"/>
     </row>
@@ -7047,11 +7093,11 @@
       <c r="A8" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="38" t="n">
+      <c r="B8" s="39" t="n">
         <v>0.072</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D8" s="10"/>
     </row>
@@ -7059,11 +7105,11 @@
       <c r="A9" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="39" t="n">
         <v>0.051</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D9" s="10"/>
     </row>
@@ -7071,11 +7117,11 @@
       <c r="A10" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="38" t="n">
+      <c r="B10" s="39" t="n">
         <v>0.044</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D10" s="10"/>
     </row>
@@ -7083,11 +7129,11 @@
       <c r="A11" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="38" t="n">
+      <c r="B11" s="39" t="n">
         <v>0.03</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D11" s="10"/>
     </row>
@@ -7095,11 +7141,11 @@
       <c r="A12" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="38" t="n">
+      <c r="B12" s="39" t="n">
         <v>0.021</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D12" s="10"/>
     </row>
@@ -7107,11 +7153,11 @@
       <c r="A13" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="38" t="n">
+      <c r="B13" s="39" t="n">
         <v>0.019</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D13" s="10"/>
     </row>
@@ -7119,11 +7165,11 @@
       <c r="A14" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="38" t="n">
+      <c r="B14" s="39" t="n">
         <v>0.016</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>761</v>
+        <v>775</v>
       </c>
       <c r="D14" s="10"/>
     </row>
@@ -7131,21 +7177,21 @@
       <c r="A15" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="39" t="n">
+      <c r="B15" s="40" t="n">
         <v>0.012</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>454</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>763</v>
+        <v>777</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="39" t="n">
+      <c r="B16" s="40" t="n">
         <v>0.0113</v>
       </c>
       <c r="C16" s="7" t="s">
@@ -7157,7 +7203,7 @@
       <c r="A17" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="39" t="n">
+      <c r="B17" s="40" t="n">
         <v>0.0106</v>
       </c>
       <c r="C17" s="7" t="s">
@@ -7169,7 +7215,7 @@
       <c r="A18" s="19" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="39" t="n">
+      <c r="B18" s="40" t="n">
         <v>0.0099</v>
       </c>
       <c r="C18" s="7" t="s">
@@ -7181,7 +7227,7 @@
       <c r="A19" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="39" t="n">
+      <c r="B19" s="40" t="n">
         <v>0.0092</v>
       </c>
       <c r="C19" s="7" t="s">
@@ -7193,7 +7239,7 @@
       <c r="A20" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="39" t="n">
+      <c r="B20" s="40" t="n">
         <v>0.0085</v>
       </c>
       <c r="C20" s="7" t="s">
@@ -7205,7 +7251,7 @@
       <c r="A21" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="39" t="n">
+      <c r="B21" s="40" t="n">
         <v>0.0078</v>
       </c>
       <c r="C21" s="7" t="s">
@@ -7217,7 +7263,7 @@
       <c r="A22" s="19" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="39" t="n">
+      <c r="B22" s="40" t="n">
         <v>0.0071</v>
       </c>
       <c r="C22" s="7" t="s">
@@ -7229,7 +7275,7 @@
       <c r="A23" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="39" t="n">
+      <c r="B23" s="40" t="n">
         <v>0.0064</v>
       </c>
       <c r="C23" s="7" t="s">
@@ -7241,7 +7287,7 @@
       <c r="A24" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="39" t="n">
+      <c r="B24" s="40" t="n">
         <v>0.0057</v>
       </c>
       <c r="C24" s="7" t="s">
@@ -7253,7 +7299,7 @@
       <c r="A25" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="39" t="n">
+      <c r="B25" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C25" s="7" t="s">
@@ -7265,7 +7311,7 @@
       <c r="A26" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="39" t="n">
+      <c r="B26" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C26" s="7" t="s">
@@ -7277,7 +7323,7 @@
       <c r="A27" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="39" t="n">
+      <c r="B27" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C27" s="7" t="s">
@@ -7289,7 +7335,7 @@
       <c r="A28" s="19" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="39" t="n">
+      <c r="B28" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C28" s="7" t="s">
@@ -7301,7 +7347,7 @@
       <c r="A29" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="39" t="n">
+      <c r="B29" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C29" s="7" t="s">
@@ -7313,7 +7359,7 @@
       <c r="A30" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="39" t="n">
+      <c r="B30" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C30" s="7" t="s">
@@ -7325,7 +7371,7 @@
       <c r="A31" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="39" t="n">
+      <c r="B31" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C31" s="7" t="s">
@@ -7337,7 +7383,7 @@
       <c r="A32" s="19" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="39" t="n">
+      <c r="B32" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C32" s="7" t="s">
@@ -7349,7 +7395,7 @@
       <c r="A33" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="39" t="n">
+      <c r="B33" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C33" s="7" t="s">
@@ -7361,7 +7407,7 @@
       <c r="A34" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="39" t="n">
+      <c r="B34" s="40" t="n">
         <v>0.003</v>
       </c>
       <c r="C34" s="7" t="s">
@@ -7373,7 +7419,7 @@
       <c r="A35" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="39" t="n">
+      <c r="B35" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C35" s="7" t="s">
@@ -7385,7 +7431,7 @@
       <c r="A36" s="19" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="39" t="n">
+      <c r="B36" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C36" s="7" t="s">
@@ -7397,7 +7443,7 @@
       <c r="A37" s="19" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="39" t="n">
+      <c r="B37" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C37" s="7" t="s">
@@ -7409,7 +7455,7 @@
       <c r="A38" s="19" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="39" t="n">
+      <c r="B38" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C38" s="7" t="s">
@@ -7421,7 +7467,7 @@
       <c r="A39" s="19" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="39" t="n">
+      <c r="B39" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C39" s="7" t="s">
@@ -7433,7 +7479,7 @@
       <c r="A40" s="19" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="39" t="n">
+      <c r="B40" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C40" s="7" t="s">
@@ -7445,7 +7491,7 @@
       <c r="A41" s="19" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="39" t="n">
+      <c r="B41" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C41" s="7" t="s">
@@ -7457,7 +7503,7 @@
       <c r="A42" s="19" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="39" t="n">
+      <c r="B42" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C42" s="7" t="s">
@@ -7469,7 +7515,7 @@
       <c r="A43" s="19" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="39" t="n">
+      <c r="B43" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C43" s="7" t="s">
@@ -7481,7 +7527,7 @@
       <c r="A44" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="39" t="n">
+      <c r="B44" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C44" s="7" t="s">
@@ -7493,7 +7539,7 @@
       <c r="A45" s="19" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="39" t="n">
+      <c r="B45" s="40" t="n">
         <v>0.0015</v>
       </c>
       <c r="C45" s="7" t="s">
@@ -11689,7 +11735,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
@@ -11970,9 +12016,141 @@
         <v>481</v>
       </c>
     </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>482</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
+        <v>483</v>
+      </c>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+    </row>
+    <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="B28" s="36" t="n">
+        <f aca="false">B6+B7</f>
+        <v>2800</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>486</v>
+      </c>
+      <c r="B29" s="33" t="n">
+        <f aca="false">12*75</f>
+        <v>900</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="B30" s="33" t="n">
+        <v>300</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
+        <v>490</v>
+      </c>
+      <c r="B31" s="34" t="n">
+        <f aca="false">B29+B30</f>
+        <v>1200</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11" t="s">
+        <v>491</v>
+      </c>
+      <c r="B32" s="34" t="n">
+        <f aca="false">B28-B31</f>
+        <v>1600</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>492</v>
+      </c>
+      <c r="B33" s="36" t="n">
+        <f aca="false">B9+B32</f>
+        <v>3100</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="B34" s="33" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>454</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>495</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A26:D26"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -12000,7 +12178,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>482</v>
+        <v>496</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -12010,7 +12188,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>483</v>
+        <v>497</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -12020,7 +12198,7 @@
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>484</v>
+        <v>498</v>
       </c>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
@@ -12030,27 +12208,27 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>485</v>
+        <v>499</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>487</v>
+        <v>501</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>488</v>
+        <v>502</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>403</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>489</v>
+        <v>503</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>490</v>
+        <v>504</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>85000</v>
@@ -12065,12 +12243,12 @@
         <v>442</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>491</v>
+        <v>505</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>492</v>
+        <v>506</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>100</v>
@@ -12085,12 +12263,12 @@
         <v>454</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>493</v>
+        <v>507</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>494</v>
+        <v>508</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>20000</v>
@@ -12105,92 +12283,92 @@
         <v>454</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>495</v>
+        <v>509</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>496</v>
-      </c>
-      <c r="B8" s="36" t="n">
+        <v>510</v>
+      </c>
+      <c r="B8" s="37" t="n">
         <v>0.25</v>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="37" t="n">
         <v>0.4</v>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="D8" s="37" t="n">
         <v>0.55</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>408</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>497</v>
+        <v>511</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>498</v>
-      </c>
-      <c r="B9" s="36" t="n">
+        <v>512</v>
+      </c>
+      <c r="B9" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="C9" s="36" t="n">
+      <c r="C9" s="37" t="n">
         <v>0.3</v>
       </c>
-      <c r="D9" s="36" t="n">
+      <c r="D9" s="37" t="n">
         <v>0.45</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>454</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>499</v>
+        <v>513</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>500</v>
-      </c>
-      <c r="B10" s="36" t="n">
+        <v>514</v>
+      </c>
+      <c r="B10" s="37" t="n">
         <v>0.4</v>
       </c>
-      <c r="C10" s="36" t="n">
+      <c r="C10" s="37" t="n">
         <v>0.45</v>
       </c>
-      <c r="D10" s="36" t="n">
+      <c r="D10" s="37" t="n">
         <v>0.5</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>408</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>501</v>
+        <v>515</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>502</v>
-      </c>
-      <c r="B11" s="36" t="n">
+        <v>516</v>
+      </c>
+      <c r="B11" s="37" t="n">
         <v>0.25</v>
       </c>
-      <c r="C11" s="36" t="n">
+      <c r="C11" s="37" t="n">
         <v>0.25</v>
       </c>
-      <c r="D11" s="36" t="n">
+      <c r="D11" s="37" t="n">
         <v>0.25</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>408</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>503</v>
+        <v>517</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>504</v>
+        <v>518</v>
       </c>
       <c r="B12" s="18" t="n">
         <v>2000</v>
@@ -12205,12 +12383,12 @@
         <v>408</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>505</v>
+        <v>519</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>506</v>
+        <v>520</v>
       </c>
       <c r="B13" s="18" t="n">
         <v>5000</v>
@@ -12225,27 +12403,27 @@
         <v>408</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>507</v>
+        <v>521</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>508</v>
-      </c>
-      <c r="B14" s="36" t="n">
+        <v>522</v>
+      </c>
+      <c r="B14" s="37" t="n">
         <v>1.3</v>
       </c>
-      <c r="C14" s="36" t="n">
+      <c r="C14" s="37" t="n">
         <v>1.6</v>
       </c>
-      <c r="D14" s="36" t="n">
+      <c r="D14" s="37" t="n">
         <v>1.9</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>408</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>509</v>
+        <v>523</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12258,7 +12436,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>510</v>
+        <v>524</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -12269,13 +12447,13 @@
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6"/>
       <c r="B17" s="6" t="s">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>487</v>
+        <v>501</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>488</v>
+        <v>502</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>403</v>
@@ -12284,7 +12462,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>511</v>
+        <v>525</v>
       </c>
       <c r="B18" s="16" t="n">
         <f aca="false">B5</f>
@@ -12305,7 +12483,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>512</v>
+        <v>526</v>
       </c>
       <c r="B19" s="16" t="n">
         <f aca="false">B7*B8</f>
@@ -12326,7 +12504,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>513</v>
+        <v>527</v>
       </c>
       <c r="B20" s="16" t="n">
         <f aca="false">B5*(1-B11)*B10*B9</f>
@@ -12347,7 +12525,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>514</v>
+        <v>528</v>
       </c>
       <c r="B21" s="16" t="n">
         <f aca="false">B12</f>
@@ -12368,7 +12546,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>515</v>
+        <v>529</v>
       </c>
       <c r="B22" s="16" t="n">
         <f aca="false">B13</f>
@@ -12389,7 +12567,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>516</v>
+        <v>530</v>
       </c>
       <c r="B23" s="31" t="n">
         <f aca="false">SUM(B18:B22)</f>
@@ -12410,7 +12588,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>517</v>
+        <v>531</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="18" t="n">
@@ -12424,7 +12602,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>518</v>
+        <v>532</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">$C$24-B23</f>
@@ -12443,17 +12621,17 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>519</v>
-      </c>
-      <c r="B26" s="37" t="n">
+        <v>533</v>
+      </c>
+      <c r="B26" s="38" t="n">
         <f aca="false">B6*(B23/B5)*B14</f>
         <v>154.202941176471</v>
       </c>
-      <c r="C26" s="37" t="n">
+      <c r="C26" s="38" t="n">
         <f aca="false">C6*(C23/C5)*C14</f>
         <v>219.494117647059</v>
       </c>
-      <c r="D26" s="37" t="n">
+      <c r="D26" s="38" t="n">
         <f aca="false">D6*(D23/D5)*D14</f>
         <v>303.650735294118</v>
       </c>
@@ -12472,7 +12650,7 @@
     </row>
     <row r="28" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>520</v>
+        <v>534</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>

</xml_diff>